<commit_message>
docs: add Template Layouts tab to slide catalog
New "Template Layouts" sheet documenting all 14 PPTX template layouts:
index, name, purpose, key placeholders, usage, and notes.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/slide_catalog.xlsx
+++ b/docs/slide_catalog.xlsx
@@ -10,11 +10,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ARS" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TXN" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ICS" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template Layouts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ARS'!$A$1:$I$80</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'TXN'!$A$1:$I$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ICS'!$A$1:$I$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Template Layouts'!$A$1:$F$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -8713,4 +8715,479 @@
   <autoFilter ref="A1:I88"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Layout Index</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Layout Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Key Placeholders</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Used For</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Cover / Intro - Slide 1</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Title slide with logo area, 3 text sections, KPI images</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>ph[0] title, ph[32] subtitle, ph[14/33/34] 3 picture slots, ph[26-31] 3 paired header+body blocks, ph[19] body text</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Opening / title slide</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>3 picture placeholders for logos/icons; 3 header+body pairs for KPI text</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Cover / Intro - Slide 2</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Minimal cover, centered title only</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ph[0] title (6.3" x 0.9")</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Simple cover / closing</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>No content areas; title is center-positioned</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Divider - Slide 2</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Section divider with subtitle bar + large content area</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>ph[0] title, ph[13] subtitle bar, ph[1] content (5.1" x 4.0")</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Section dividers between modules</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Left-aligned layout; content area can hold bullets or overview text</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Divider - Slide 3</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Minimal section divider with subtitle bar</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>ph[0] title, ph[13] subtitle bar</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Section dividers (minimal)</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Full-width title; no content area beyond subtitle</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Analysis - Slide 1 (Chart + 2 Text)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Chart on left, 2 header+body text sections on right</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>ph[0] title, ph[13] subtitle, ph[14] picture (5.5" x 3.4" left), ph[26/19] top header+body, ph[27/28] bottom header+body</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>screenshot_kpi slides (chart + KPI callouts)</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Right side has 2 independent text zones for insights/KPIs</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Analysis - Slide 2 (Chart + 1 Text)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Chart on left, single tall text section on right</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>ph[0] title, ph[13] subtitle, ph[14] picture (5.5" x 3.4" left), ph[26] header, ph[19] body (5.7" x 4.0" right)</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>screenshot_kpi slides (chart + narrative)</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Right body is 4" tall -- good for longer narratives or bullet lists</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Analysis - Slide 3 - Split</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Two equal content areas side-by-side</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>ph[0] title, ph[13] subtitle, ph[14] left (5.8" x 4.3"), ph[1] right (5.8" x 4.3")</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>multi_screenshot (2 charts side-by-side)</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Both zones are generic OBJECT placeholders; can hold images or text</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Analysis - Slide 4 - Split</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>6-cell KPI grid (3 header+body pairs per column)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>ph[0] title, ph[13] subtitle, ph[26-30] left 3 pairs, ph[32-36] right 3 pairs</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>KPI summary / data grid slides</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>12 text placeholders total; designed for structured KPI readouts</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Analysis - Slide 5 - Thirds</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>6-cell grid (3 columns x 2 rows of content blocks)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>ph[0] title, ph[13] subtitle, ph[1/15/16] top row, ph[17/19/20] bottom row</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Multi-chart grids, comparison panels</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Each cell is 3.6" x 2.1"; all OBJECT type (images or text)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Analysis - Slide 6 - Main</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Full-width single content area (the workhorse screenshot layout)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>ph[0] title, ph[13] subtitle, ph[1] content (11.7" x 4.3")</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>screenshot (single full-width chart)</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Most common layout; used for any single chart/image</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Analysis - Slide 7 - Stacked Two</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>2 rows: each has text on left + 3 pictures on right</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>ph[0] title, ph[15/35] row headers, ph[19/36] row body, ph[29-31] top 3 pics, ph[32-34] bottom 3 pics</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Before/after comparisons, multi-image galleries</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>6 picture placeholders (2.1" x 1.8" each); good for small chart grids</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Analysis - Slide 8 - Blank</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Blank slide with right-aligned title</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>ph[0] title (6.4" x 1.6", right side)</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Custom-built slides, freeform content</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>No content placeholders; shapes must be added programmatically</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Analysis - Slide 11 - Header1</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Pure background / decorative header</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>(no placeholders)</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Visual separator, background-only</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>No usable placeholders; purely decorative</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Analysis - Slide 11 - Header2</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Background header with footer/slide number</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>ph[11] footer, ph[12] slide number</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Mailer summaries, wide charts (custom positioning)</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>No title/content placeholders; content placed via freeform shapes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F15"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Slide Types reference tab to catalog
New "Slide Types" sheet mapping each slide type to its layout,
when to use it, content zones, and real examples from all pipelines.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/slide_catalog.xlsx
+++ b/docs/slide_catalog.xlsx
@@ -10,13 +10,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ARS" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TXN" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ICS" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template Layouts" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slide Types" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template Layouts" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ARS'!$A$1:$I$80</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'TXN'!$A$1:$I$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ICS'!$A$1:$I$88</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Template Layouts'!$A$1:$F$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Slide Types'!$A$1:$F$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Template Layouts'!$A$1:$F$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -9741,6 +9743,359 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Slide Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Layout Index</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Layout Name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>When To Use</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Content Zones</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Examples</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>chart_narrative</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Analysis - Slide 2 (Chart + 1 Text)</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Any chart that needs explanatory text -- trend lines, donuts, scatters, funnels, waterfalls</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Chart (5.5" x 3.4" left) + header + tall body (5.7" x 4.0" right)</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>DCTR-1 trend, A7.8 funnel, A11.1 waterfall, ax08 source donut, ax29 milestones</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>chart_kpi</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Analysis - Slide 1 (Chart + 2 Text)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Charts with 2 KPI callout zones -- rates, snapshots, impact metrics with headline numbers</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Chart (5.5" x 3.4" left) + top header+body + bottom header+body (right)</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>DCTR-3 snapshot, A8.3 Reg E snapshot, A9.1 attrition rate, A9.9-A9.11 impact KPIs</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>comparison</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Analysis - Slide 3 - Split</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Natural A-vs-B content -- Personal vs Business, Open vs Closed, DM vs REF, rank vs change</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Left content (5.8" x 4.3") + right content (5.8" x 4.3")</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>DCTR-4/5 personal vs business, A9.13 ARS vs non-ARS, ax14 age comparison, REF-4 one-time vs repeat</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>multi_screenshot</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Analysis - Slide 3 - Split</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Merged chart pairs -- two related charts that tell one story side by side</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Left content (5.8" x 4.3") + right content (5.8" x 4.3")</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>A7.6a trajectory+segments, A7.7 historical vs TTM, A8.5 opportunity, A9.3 open vs closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>kpi_grid</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Analysis - Slide 4 - Split</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Pure KPI summary slides -- structured readouts with 6 metric cells</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>6 cells: 3 header+body pairs per column (left 3, right 3)</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>A7.10c branch KPIs, A8.12 Reg E summary, ax01/02 ICS summary, ax22 activity, REF-8 overview</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>grid_thirds</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Analysis - Slide 5 - Thirds</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Multi-panel charts -- 3+ small charts or comparison panels in a grid</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>6 cells: 3 columns x 2 rows (each 3.6" x 2.1")</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>MCC 3-panel comparison, portfolio scorecard bullet gauges</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>screenshot</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Analysis - Slide 6 - Main</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Data-dense charts that need full width -- heatmaps, long merchant lists, many-branch bars</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Full-width content (11.7" x 4.3")</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>DCTR-8 summary, DCTR-9 heatmap, top-25 merchants, branch rank bars, cohort heatmaps</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>section_text</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Divider - Slide 2</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Text-only slides -- conclusions, section intros with explanatory content</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Title + subtitle bar + large text content area (5.1" x 4.0")</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>S6-S8 conclusions, section overview text</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>wide_custom</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Analysis - Slide 11 - Header2</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Dense matrices needing freeform positioning -- wide heatmaps, custom mailer layouts</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>No content placeholders; shapes added programmatically</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>A7.10a branch matrix, A8.4a branch Reg E matrix, mailer monthly summaries</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>data_only</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>(no PPTX slide)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Excel-only tables and data engine steps -- no visual chart, no slide generated</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>N/A -- data appears in Excel report only</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>MCC tables, monthly movers, competitor detection, dormant lists, overview tables</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
docs(catalog): add File Paths, Data Sources, and M Drive Paths tabs
Three new reference tabs in the slide catalog workbook:
- File Paths (90 rows): all code files by category
- Data Sources (13 rows): input data types per pipeline
- M Drive Paths (11 rows): Windows M: drive structure

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/slide_catalog.xlsx
+++ b/docs/slide_catalog.xlsx
@@ -12,6 +12,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ICS" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slide Types" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template Layouts" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Sources" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M Drive Paths" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="File Paths" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ARS'!$A$1:$I$80</definedName>
@@ -19,6 +22,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ICS'!$A$1:$I$88</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Slide Types'!$A$1:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Template Layouts'!$A$1:$F$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Data Sources'!$A$1:$F$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'M Drive Paths'!$A$1:$D$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'File Paths'!$A$1:$D$91</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -10563,4 +10569,2783 @@
   <autoFilter ref="A1:F15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Source Location</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Format</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Key Columns</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>ODD (raw)</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>M:\CSM-Source\Folder\ClientID_ODDD*.xlsx</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Excel (.xlsx)</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Account #, Date Opened, Date Closed, Stat Code, Prod Code, Branch, DOB, Balance fields</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Copied by retrieve_all() to retrieve_dir/CSM/YYYY.MM/ClientID/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>ODD (formatted)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>watch_root\CSM\YYYY.MM\ClientID\*-formatted.xlsx</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Excel (.xlsx)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>All raw cols + Total Spend, Total Swipes, Avg Monthly, Account Age, Holder Age, Response Grouping, Segmentation</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Created by format_odd() 7-step pipeline; scan_ready_files() prefers these</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Client Config</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>M:\ARS\Config\clients_config.json  OR  config/clients_config.json</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>JSON</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>ClientID, DataStartDate, ICRate, NSF_OD_Fee, EligibleStatusCodes, BranchMapping</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Per-client overrides; falls back to defaults</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>ARS Config</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>ars_config.json (project root or ARS_CONFIG_PATH env)</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>JSON</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>paths (ars_base, watch_root, retrieve_dir), csm_sources, pipeline settings</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Loaded by ARSSettings; env vars with ARS_ prefix override</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Transaction CSV</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>User-provided or auto-discovered near ODD file</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>CSV/TXT (tab-delimited)</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>merchant_name, amount, primary_account_num, transaction_date, mcc_code, business_flag, year_month</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>50+ column aliases auto-resolved by resolve_columns(); 13-col standard layout</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>ODD (for segments)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Via --odd CLI flag or Settings.odd_file</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Excel (.xlsx)</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Account #, Segmentation cols (MmmYY Seg), ICS Account, generation, tenure, balance_tier</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Optional; enables M11 demographics, segment filters (ARS responders, ICS accounts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Transaction Dir</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Settings.transaction_dir (year-folder layout)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Directory of CSVs</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>YYYY/MM/*.csv files; auto-selects most recent 12 months</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Alternative to single file; V4 multi-month mode</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>ICS</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>ICS Excel</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>User-provided or M: drive</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Excel (.xlsx)</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Account #, ICS Account (Yes/No), ICS Source (REF/DM/Both), Stat Code, Prod Code, Branch, Balance, Date Opened/Closed</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Core input; L12M monthly columns auto-discovered (MmmYY pattern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>ICS</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Referral Data</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Same ICS Excel or separate referral file</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Excel (.xlsx)</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Referring Account, Referred Account, Referral Date, Referral Code, Branch</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Used by referral pipeline (REF-1 to REF-8); requires code_decoder for code classification</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>ICS</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Revenue Workbook</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>ICS directory or config path</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Excel (.xlsx)</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Account #, Monthly Interchange, Annual Revenue</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Optional; enables revenue impact analyses (ax39, ax65, ax66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>ICS</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Benchmarks</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>config/benchmarks.json</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>JSON</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>debit_penetration_rate, active_card_rate, avg_annual_spend_per_card, direct_mail_response_rate</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Industry benchmarks for comparison analyses</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>PPTX Template</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>packages/shared/src/shared/deck/template/Template12.25.pptx</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>PowerPoint (.pptx)</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>14 layouts (cover, divider, chart+text, split, grid, blank, etc.)</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Identical copies in ars_analysis and ics_toolkit packages</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Platform Config</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>config/platform.yaml</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>YAML</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>base_output_dir, m_drive_path, chart_theme, per-pipeline enabled/settings</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Top-level orchestrator config</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F14"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="55" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Path</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Read/Write</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Used By</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>M:\ARS\</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>ARS base directory</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>R/W</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>All ARS operations</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>M:\ARS\Ready for Analysis\CSM\YYYY.MM\ClientID\</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Formatted ODD files (watch_root)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>R/W</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>scan, analyze, batch</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>M:\ARS\Incoming\ODDD Files\CSM\YYYY.MM\ClientID\</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Raw ODD files (retrieve_dir)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>R/W</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>retrieve_all()</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>M:\ARS\Presentations\Presentation Excels\</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Output Excel reports</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Write</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>excel_formatter, batch</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>M:\ARS\Presentations\Presentation Excels\Archive\</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Archived previous reports</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Write</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>batch (auto-archive)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>M:\ARS\Presentations\Template12.25.pptx</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>PPTX template (runtime)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>deck_builder</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>M:\ARS\Scripts\Config\</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Runtime config directory</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>ARSSettings</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>M:\ARS\Config\clients_config.json</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Master client config</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Pipeline context, per-client overrides</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>M:\ARS\Logs\</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Pipeline log files</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Write</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>All pipelines</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>M:\CSM-Source\{CSMName}\</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>CSM source directories (per ars_config.json csm_sources)</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>retrieve_all()</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>M:\ICS\Config\clients_config.json</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>ICS client config fallback</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>ICS pipeline</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D12"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D91"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Package</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>File Path</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>ars_analysis</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>ars_analysis/config.py</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>PathsConfig, CSMSourcesConfig, PipelineConfig, ARSSettings (loads ars_config.json)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>shared/config.py</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>PlatformConfig (base_output_dir, m_drive_path, chart_theme, template_pptx, pipelines)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>txn_analysis</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>txn_analysis/settings.py</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Settings (data_file, odd_file, output_dir, charts, outputs, segments)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>ics_toolkit</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>ics_toolkit/settings.py</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>AppendSettings, AnalysisSettings, ReferralSettings</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>root</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>config/platform.yaml</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Top-level platform config (per-pipeline settings)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>root</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>config/clients_config.json</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Master client config (DataStartDate, ICRate, NSF_OD_Fee, BranchMapping, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Config</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>root</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>config/benchmarks.json</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Industry benchmarks (debit penetration, active card rate, avg spend)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Data Loader</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>shared/data_loader.py</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>load_oddd(), load_tran(), load_odd(), _read_file() (auto-detect xlsx/xls/csv)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Data Loader</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>ars_analysis</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>ars_analysis/pipeline/steps/load.py</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Load ODD file for ARS pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Data Loader</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>txn_analysis</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>txn_analysis/data_loader.py</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>load_data(), load_odd(), merge_odd(), _apply_merchant_consolidation(), _derive_year_month()</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Data Loader</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>ics_toolkit</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>ics_toolkit/analysis/data_loader.py</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>load_data(), _normalize_strings(), _parse_dates(), _coerce_numerics(), discover L12M cols</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Data Loader</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>ics_toolkit</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>ics_toolkit/referral/data_loader.py</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Referral-specific data loading and normalization</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Retrieve/Format</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>ars_analysis</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>ars_analysis/pipeline/steps/retrieve.py</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>retrieve_all() -- copy ODD from CSM M: drive sources to retrieve_dir/CSM/YYYY.MM/ClientID/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Retrieve/Format</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>shared/format_odd.py</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>format_odd() 7-step pipeline (PYTD drop, totals, PIN+Sig, age, response, segmentation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Retrieve/Format</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>ars_analysis</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>ars_analysis/pipeline/steps/format.py</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>format_all() -- batch format from retrieve_dir to watch_root</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Retrieve/Format</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>ars_analysis</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>ars_analysis/pipeline/steps/scan.py</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>scan_ready_files(), _pick_best_file() (prefers *-formatted.xlsx), available_months/csms</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Column Mapping</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>txn_analysis</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>txn_analysis/column_map.py</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>COLUMN_ALIASES (50+ header variations), resolve_columns(), REQUIRED/OPTIONAL_COLUMNS</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Column Mapping</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>ics_toolkit</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>ics_toolkit/analysis/column_map.py</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>resolve_columns(), validate_columns(), discover_l12m_columns()</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Column Mapping</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>ics_toolkit</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>ics_toolkit/referral/column_map.py</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Referral column normalization</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Reference Data</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>txn_analysis</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>txn_analysis/competitor_patterns.py</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>COMPETITOR_MERCHANTS (7 categories, 3-tier matching), FINANCIAL_MCC_CODES, classify_merchant()</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Reference Data</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>txn_analysis</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>txn_analysis/segments.py</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>extract_responder_accounts(), extract_ics_accounts(), build_segment_filters()</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Reference Data</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>txn_analysis</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>txn_analysis/formatting.py</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>excel_number_format(), is_percentage_column(), is_grand_total_row()</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Reference Data</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>ics_toolkit</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>ics_toolkit/referral/code_decoder.py</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Referral code decoding and classification</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Reference Data</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>ics_toolkit</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>ics_toolkit/referral/scoring.py</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Referral scoring weights and calculations</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Deck Builder</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>shared/deck/__init__.py</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Re-exports: DeckBuilder, SlideContent, build_deck_from_results</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Deck Builder</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>shared/deck/engine.py</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>DeckBuilder class + SlideContent dataclass (extracted reusable engine)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Deck Builder</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>shared/deck/universal.py</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>build_deck_from_results() -- universal builder for TXN/ICS/Attrition</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Deck Builder</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>ars_analysis</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>ars_analysis/output/deck_builder.py</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>ARS-specific deck builder (500+ lines, section ordering, mailer logic)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Deck Builder</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>ics_toolkit</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>ics_toolkit/analysis/exports/deck_builder.py</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>ICS analysis deck builder</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Deck Builder</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>ics_toolkit</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>ics_toolkit/analysis/exports/pptx.py</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>ICS PPTX export helpers</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Deck Builder</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>ics_toolkit</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>ics_toolkit/analysis/exports/kpi_slides.py</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>ICS KPI slide builder</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Deck Builder</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>ics_toolkit</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>ics_toolkit/referral/exports/pptx.py</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>ICS referral deck builder</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Deck Builder</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>txn_analysis</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>txn_analysis/exports/pptx_report.py</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>TXN PPTX report (charts-only deck)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Template</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>shared/deck/template/Template12.25.pptx</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Shared PPTX template (14 layouts) -- canonical copy</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Template</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>ars_analysis</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>ars_analysis/output/template/Template12.25.pptx</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>ARS copy of template</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Template</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>ics_toolkit</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>ics_toolkit/templates/Template12.25.pptx</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>ICS copy of template</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Excel Export</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>shared/excel.py</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Shared Excel helpers (formatting, styles)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Excel Export</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>ars_analysis</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>ars_analysis/output/excel_formatter.py</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>ARS Excel report (Summary sheet, KPI extraction, per-section tabs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Excel Export</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>ics_toolkit</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>ics_toolkit/analysis/exports/excel.py</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>ICS analysis Excel report</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Excel Export</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>ics_toolkit</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>ics_toolkit/referral/exports/excel.py</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>ICS referral Excel report</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Excel Export</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>txn_analysis</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>txn_analysis/exports/excel_report.py</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>TXN Excel report (cover, TOC, per-analysis sheets, chart embeds)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Charts</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>shared/charts.py</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Shared chart utilities (chart_figure context manager, style isolation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Charts</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>ars_analysis</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>ars_analysis/charts/__init__.py</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>ARS chart registry + style</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Charts</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>ars_analysis</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>ars_analysis/charts/guards.py</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>ARS matplotlib leak guards</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Charts</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>txn_analysis</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>txn_analysis/charts/__init__.py</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>TXN chart registry (CHART_REGISTRY dict), create_charts(), render_chart_png()</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Charts</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>txn_analysis</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>txn_analysis/charts/builders.py</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>TXN chart primitives (lollipop, donut, heatmap, grouped_bar, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Charts</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>txn_analysis</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>txn_analysis/charts/theme.py</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>TXN chart theme + add_source_footer()</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Charts</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>txn_analysis</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>txn_analysis/charts/{overall,personal,business,mcc,competitor,trends,recurring,scorecard}.py</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>TXN per-section chart functions</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Charts</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>ics_toolkit</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>ics_toolkit/analysis/charts/__init__.py</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>ICS chart registry</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Charts</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>ics_toolkit</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>ics_toolkit/analysis/charts/renderer.py</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>ICS chart renderer (PNG export)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Charts</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>ics_toolkit</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>ics_toolkit/analysis/charts/{summary,source,dm_source,activity,demographics,cohort,performance,portfolio,persona,strategic}.py</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>ICS per-section chart functions</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Charts</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>ics_toolkit</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>ics_toolkit/referral/charts/{top_referrers,branch_density,code_health,staff_multipliers,emerging_referrers}.py</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>ICS referral chart functions</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>ars_analysis</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>ars_analysis/analytics/registry.py</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>ARS module registry (ABC + @register)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>ars_analysis</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>ars_analysis/analytics/overview/{stat_codes,product_codes,eligibility}.py</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Overview: A1, A1b, A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>ars_analysis</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>ars_analysis/analytics/dctr/{penetration,trends,branches,funnel,overlays,_helpers}.py</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>DCTR: DCTR-1 to 16, A7.x (26 slides)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>ars_analysis</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>ars_analysis/analytics/rege/{status,branches,dimensions,_helpers}.py</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Reg E: A8.x (13 slides)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>ars_analysis</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>ars_analysis/analytics/attrition/{rates,dimensions,impact,_helpers}.py</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>Attrition: A9.x (13 slides)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>ars_analysis</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>ars_analysis/analytics/value/analysis.py</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>Value: A11.1, A11.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>ars_analysis</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>ars_analysis/analytics/mailer/{reach,response,impact,insights,cohort,_helpers}.py</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>Mailer: A12-A15 (dynamic per month)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>ars_analysis</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>ars_analysis/analytics/insights/{synthesis,conclusions,effectiveness,dormant,branch_scorecard,_data}.py</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>Insights: S1-S8</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>ics_toolkit</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>ics_toolkit/analysis/analyses/{summary,source,dm_source,ref_source,demographics,activity,cohort,performance,portfolio,persona,strategic}.py</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>ICS: 82 chart slides across 12 sections</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>ics_toolkit</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>ics_toolkit/referral/analyses/{overview,top_referrers,branch_density,code_health,emerging_referrers,dormant_referrers,staff_multipliers,onetime_vs_repeat}.py</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>Referral: REF-1 to REF-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>txn_analysis</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>txn_analysis/analyses/{overall,personal,business,mcc,financial_services,interchange,member_segments}.py</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>TXN: M1-M4, M7-M8, M10</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>txn_analysis</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>txn_analysis/analyses/{competitor_detect,competitor_metrics,competitor_segment,competitor_threat}.py</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>TXN: M6 competitor</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>txn_analysis</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>txn_analysis/analyses/{trends_rank,trends_growth,trends_consistency,trends_cohort,trends_movers}.py</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>TXN: M5 trends</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>txn_analysis</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>txn_analysis/analyses/{recurring,scorecard,spending_behavior,time_patterns}.py</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>TXN: M9, M15, behavioral</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>platform_app</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>platform_app/orchestrator.py</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>Central orchestrator + _ensure_deck() fallback</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>ars_analysis</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>ars_analysis/pipeline/runner.py</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>ARS pipeline runner (load -&gt; subset -&gt; analyze -&gt; generate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>ars_analysis</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>ars_analysis/pipeline/context.py</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>ARS PipelineContext dataclass</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>ars_analysis</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>ars_analysis/pipeline/batch.py</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>ARS batch runner (run_batch for 300+ clients)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>ars_analysis</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>ars_analysis/runner.py</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>ARS CLI entry point</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>ics_toolkit</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>ics_toolkit/analysis/pipeline.py</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>ICS analysis pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>ics_toolkit</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>ics_toolkit/referral/pipeline.py</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>ICS referral pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>ics_toolkit</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>ics_toolkit/runner.py</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>ICS CLI entry point</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>txn_analysis</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>txn_analysis/pipeline.py</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>TXN pipeline (load -&gt; analyze -&gt; chart -&gt; export)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>txn_analysis</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>txn_analysis/runner.py</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>TXN CLI entry point</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>platform_app</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>platform_app/pages/pipeline_ars.py</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>Streamlit ARS pipeline page</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>platform_app</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>platform_app/pages/pipeline_txn.py</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>Streamlit TXN pipeline page</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>platform_app</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>platform_app/pages/pipeline_ics.py</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>Streamlit ICS pipeline page</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>platform_app</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>platform_app/pages/pipeline_attrition.py</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>Streamlit Attrition pipeline page</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Script</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>root</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>run.bat</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>4-step pipeline: retrieve -&gt; format -&gt; batch -&gt; streamlit</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>Script</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>root</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>run_batch.bat</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>Headless batch runner</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Script</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>root</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>dashboard.bat</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>Launch Streamlit UI only</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>Script</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>root</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>setup.bat</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>Environment setup (uv install)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>root</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>tests/e2e_data/1200_Test CU_2026.02.xlsx</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>Synthetic ARS ODD (20 accounts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>root</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>tests/e2e_data/8888_transactions.csv</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>Synthetic TXN (35 transactions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>root</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>tests/e2e_data/9999_ICS_2026.01.xlsx</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>Synthetic ICS (80 accounts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>root</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>tests/e2e_data/generate_fixtures.py</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>E2E fixture generator script</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>Catalog</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>root</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>docs/slide_catalog.py</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>This file -- generates the catalog Excel</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>Catalog</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>root</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>docs/slide_catalog.xlsx</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>Generated workbook (all tabs)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D91"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(catalog): add Field Names and Cross-Pipeline Fields tabs
Two new reference tabs in the slide catalog workbook:
- Field Names (101 rows): every column across ODD/TXN/ICS with aliases,
  required flag, type, source, and notes
- Cross-Pipeline Fields (19 rows): shows which ODD fields feed into
  ARS, TXN, and ICS pipelines with per-pipeline purpose

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/slide_catalog.xlsx
+++ b/docs/slide_catalog.xlsx
@@ -15,6 +15,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Sources" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M Drive Paths" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="File Paths" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Names" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cross-Pipeline Fields" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ARS'!$A$1:$I$80</definedName>
@@ -25,6 +27,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Data Sources'!$A$1:$F$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'M Drive Paths'!$A$1:$D$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'File Paths'!$A$1:$D$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Field Names'!$A$1:$H$102</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Cross-Pipeline Fields'!$A$1:$G$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -4090,6 +4094,698 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ODD Field</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Used by ARS</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Used by TXN</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Used by ICS</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ARS Purpose</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>TXN Purpose</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>ICS Purpose</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Acct Number</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Yes (merge key)</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Yes (merge key)</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr"/>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Joins TXN rows to ODD demographics</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Joins ICS append to ODD rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Stat Code</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Subset filtering, eligibility</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Account status filtering</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Product Code / Prod Code</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Eligibility, product analysis</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr"/>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Product-level ICS analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Date Opened</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Yes (merge)</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>L12M filtering, age calc, attrition</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Account tenure</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Age calc, account age</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Date Closed</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Yes (merge)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Yes (optional)</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Open/closed split, attrition</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Account status</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Open/closed filtering</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Avg Bal</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Yes (merge)</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Yes (optional)</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Balance categorization</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Balance tier binning</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Balance analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Business?</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Yes (merge)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Personal/business split</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Business flag on TXN rows</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>P/B segmentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Debit?</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Yes (merge)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>DCTR, Reg E, Value modules</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Debit flag on TXN rows</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Debit account filtering</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Yes (merge)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Branch-level DCTR, attrition</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Branch on TXN rows</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Branch-level ICS analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Account Holder Age</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Yes (merge)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Demographics, age categories</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Generation cohort derivation</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>DOB</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Age computation in format_odd</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr"/>
+      <c r="G12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>MmmYY Spend</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Mailer impact, trends</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr"/>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>L12M activity analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>MmmYY Swipes</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Mailer impact, trends</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr"/>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>L12M activity analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>MmmYY Mail</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Mailer module, offer counting</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr"/>
+      <c r="G15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>MmmYY Resp</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Yes (segments)</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Mailer module, segmentation</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Responder segment filters</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>MmmYY Reg E Code</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Reg E module analysis</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr"/>
+      <c r="G17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>ICS Account</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Yes (segments)</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>ICS segment filters</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Core analysis column</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>ICS Source / Source</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr"/>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>REF/DM/Both source analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Curr Bal</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="3" t="inlineStr"/>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Balance-tier analysis</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G20"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -13348,4 +14044,4097 @@
   <autoFilter ref="A1:D91"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H102"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Pipeline</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Field Name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Aliases</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Acct Number</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Raw Excel</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Primary key for cross-pipeline merges</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Stat Code</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Status Code, StatCode, Stat_Code, Account Status</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Raw Excel</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Account status (O=Open, C=Closed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Product Code</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Prod Code, ProdCode, Prod_Code</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Raw Excel</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Product type identifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Date Opened</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>DateOpened, Date_Opened, Open Date</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>datetime</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Raw Excel</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Account open date</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Date Closed</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>DateClosed, Date_Closed, Close Date</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>datetime</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Raw Excel</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Account close date (NaT if open)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Avg Bal</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Balance, Current Balance, Cur Bal, AvgBal, Avg_Bal, Average Balance</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Raw Excel</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Average balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Raw Excel</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Branch identifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Business?</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Business, BusinessFlag, Business Flag</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Raw Excel</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Personal vs business flag</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Debit?</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Debit, DC Indicator, DC_Indicator, DebitCard, Debit Card</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Raw Excel</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Debit card indicator (YES/Y/D/DC/DEBIT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>DOB</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>datetime</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Raw Excel</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Date of birth (used to compute age)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Mailable?</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Raw Excel</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Eligibility flag for mailers</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>MmmYY PIN $</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>e.g. Jan25 PIN $</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Raw Excel</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>PIN debit dollar amount per month</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>MmmYY Sig $</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>e.g. Jan25 Sig $</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Raw Excel</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Signature debit dollar amount per month</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>MmmYY PIN #</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>e.g. Jan25 PIN #</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Raw Excel</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>PIN debit transaction count per month</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>MmmYY Sig #</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>e.g. Jan25 Sig #</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Raw Excel</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Signature debit transaction count per month</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>MmmYY MTD</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>e.g. Jan25 MTD</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Raw Excel</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Month-to-date items</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>MmmYY OD Limit</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>e.g. Jan25 OD Limit</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Raw Excel</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Overdraft limit per month</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>MmmYY Reg E Code</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>e.g. Jan25 Reg E Code</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Raw Excel</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Reg E status code per month</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>MmmYY Reg E Desc</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>e.g. Jan25 Reg E Desc</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Raw Excel</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Reg E description per month</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>MmmYY Mail</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>e.g. Jan25 Mail</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Raw Excel</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Mailer segment code per month</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>MmmYY Resp</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>e.g. Jan25 Resp</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Raw Excel</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Response segment code per month</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>MmmYY Spend</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>e.g. Jan25 Spend</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>format_odd</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>PIN $ + Sig $ combined per month</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>MmmYY Swipes</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>e.g. Jan25 Swipes</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>format_odd</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>PIN # + Sig # combined per month</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Total Spend</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>format_odd</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Sum of all monthly Spend</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Total Swipes</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>format_odd</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>Sum of all monthly Swipes</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Total Items</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>format_odd</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>Sum of all monthly MTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>last 3-mon spend</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>format_odd</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>Last 3 months cumulative spend</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>last 3-mon swipes</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>format_odd</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Last 3 months cumulative swipes</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Last 3-mon Items</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>format_odd</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>Last 3 months cumulative items</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>last 12-mon spend</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>format_odd</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>Last 12 months cumulative spend</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>last 12-mon swipes</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr"/>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>format_odd</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>Last 12 months cumulative swipes</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Last 12-mon Items</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>format_odd</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>Last 12 months cumulative items</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>MonthlySpend12</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr"/>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>format_odd</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>12-month avg monthly spend</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>MonthlySwipes12</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>format_odd</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>12-month avg monthly swipes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>MonthlyItems12</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr"/>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>format_odd</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>12-month avg monthly items</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>MonthlySpend3</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>format_odd</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>3-month avg monthly spend</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>MonthlySwipes3</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr"/>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>format_odd</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>3-month avg monthly swipes</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>MonthlyItems3</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr"/>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>format_odd</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>3-month avg monthly items</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>SwipeCat12</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr"/>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>format_odd</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>12-month swipe tier (Non-user, 1-5, 6-10, 11-20, 21-40, 41+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>SwipeCat3</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr"/>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>format_odd</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>3-month swipe tier</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Account Holder Age</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr"/>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>format_odd</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>Years from DOB to report date</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Account Age</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr"/>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>format_odd</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>Years from Date Opened to close/report date</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t># of Offers</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr"/>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>format_odd</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>Count of non-null Mail columns</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t># of Responses</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr"/>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>format_odd</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>Count of non-null Resp columns (excl NU 1-4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Response Grouping</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr"/>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>format_odd</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>No Offer / Non-Responder / SO-SR / MO-SR / MR</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>MmmYY Segmentation</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>e.g. Jan25 Segmentation</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>format_odd</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>Control / Non-Responder / Responder per month</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>ICS Account</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr"/>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>ICS append</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>Yes / No (appended by ICS pipeline)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>ICS Source</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr"/>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>ICS append</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>REF / DM / Both / empty</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>merchant_name</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>merchantname, merchant, merch_name, description, payee, vendor, ...</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>Merchant/payee name (12 aliases)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>transaction_amount, txn_amount, amt, debit_amount, purchase_amount, ...</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>Transaction dollar amount (11 aliases)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>primary_account_num</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>account_number, acct_num, card_number, pan, member_number, ...</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>Account identifier (18 aliases)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>transaction_date</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>trans_date, txn_date, date, posting_date, settlement_date, ...</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>datetime</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>Transaction date (12 aliases)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>mcc_code</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>mcccode, mcc, merchant_category_code, sic_code, sic</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>Merchant Category Code (7 aliases)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>business_flag</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>businessflag, business, is_business, account_type</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>Business account indicator (6 aliases)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>year_month</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>yearmonth, ym</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>Pre-computed YYYY-MM period</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>V4 Positional</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>transaction_type</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr"/>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>Tab file col 3</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>Transaction type code</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>V4 Positional</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>terminal_location_1</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr"/>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>Tab file col 7</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>Terminal location line 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>V4 Positional</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>terminal_location_2</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr"/>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>Tab file col 8</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>Terminal location line 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>V4 Positional</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>terminal_id</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr"/>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>Tab file col 9</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>Terminal identifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>V4 Positional</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>merchant_id</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr"/>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>Tab file col 10</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>Merchant identifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>V4 Positional</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>institution</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr"/>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>Tab file col 11</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>Issuing institution</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>V4 Positional</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>card_present</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr"/>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>Tab file col 12</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>Card-present indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>V4 Positional</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>transaction_code</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr"/>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>Tab file col 13</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>Transaction code</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>merchant_consolidated</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr"/>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>data_loader</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>Standardized merchant name via rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>year_month</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>(if not in CSV)</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>data_loader</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>YYYY-MM derived from transaction_date</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>is_partial_month</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr"/>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>data_loader</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>True if last month has &lt;90% day coverage</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>source_file</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr"/>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>data_loader</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>Originating CSV filename</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>generation</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr"/>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>ODD merge</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>Gen Z / Millennial / Gen X / Boomer / Silent</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>balance_tier</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr"/>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>ODD merge</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t>Low / Medium / High / Very High</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>tenure_years</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr"/>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>ODD merge</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>Years since account opened</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>ICS</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>ICS Account</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>ICS Accounts, Ics Account, ICS_Account, IcsAccount</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>ICS account flag (Yes/No)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>ICS</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>Stat Code</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>StatCode, Stat_Code, Status Code</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>Account status code</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>ICS</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>Debit?</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>Debit, DebitCard, Debit Card</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="H74" s="3" t="inlineStr">
+        <is>
+          <t>Debit card indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>ICS</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>Business?</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>Business, BusinessFlag, Business Flag</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="H75" s="3" t="inlineStr">
+        <is>
+          <t>Personal vs business flag</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>ICS</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>Date Opened</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>DateOpened, Date_Opened, Open Date</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>datetime</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>Account open date</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>ICS</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>Prod Code</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>ProdCode, Prod_Code, Product Code</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>Product code</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>ICS</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr"/>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>Branch identifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>ICS</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr"/>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G79" s="3" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="H79" s="3" t="inlineStr">
+        <is>
+          <t>ICS source (REF/DM/Both)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>ICS</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>Curr Bal</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>CurrBal, Curr_Bal, Current Balance</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>Current balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>ICS</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>Date Closed</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>DateClosed, Date_Closed, Close Date</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
+          <t>datetime</t>
+        </is>
+      </c>
+      <c r="G81" s="3" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="H81" s="3" t="inlineStr">
+        <is>
+          <t>Account close date</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>ICS</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>Avg Bal</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>AvgBal, Avg_Bal, Average Balance, AvgColBal</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="G82" s="3" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="H82" s="3" t="inlineStr">
+        <is>
+          <t>Average balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>ICS</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>L12M</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>MmmYY Swipes</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>regex: ^[A-Z][a-z]{2}\d{2} Swipes$</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="G83" s="3" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="H83" s="3" t="inlineStr">
+        <is>
+          <t>Monthly swipe count (e.g. Feb24 Swipes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>ICS</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>L12M</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>MmmYY Spend</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>regex: ^[A-Z][a-z]{2}\d{2} Spend$</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>Monthly spend (e.g. Feb24 Spend)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>ICS</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>Total L12M Swipes</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr"/>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t>utils.py</t>
+        </is>
+      </c>
+      <c r="H85" s="3" t="inlineStr">
+        <is>
+          <t>Sum of all MmmYY Swipes columns</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>ICS</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>Total L12M Spend</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr"/>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F86" s="3" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="G86" s="3" t="inlineStr">
+        <is>
+          <t>utils.py</t>
+        </is>
+      </c>
+      <c r="H86" s="3" t="inlineStr">
+        <is>
+          <t>Sum of all MmmYY Spend columns</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>ICS</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>Active in L12M</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr"/>
+      <c r="E87" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F87" s="3" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="G87" s="3" t="inlineStr">
+        <is>
+          <t>utils.py</t>
+        </is>
+      </c>
+      <c r="H87" s="3" t="inlineStr">
+        <is>
+          <t>True if Total L12M Swipes &gt; 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>ICS</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>Opening Month</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr"/>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F88" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G88" s="3" t="inlineStr">
+        <is>
+          <t>utils.py</t>
+        </is>
+      </c>
+      <c r="H88" s="3" t="inlineStr">
+        <is>
+          <t>YYYY-MM from Date Opened</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>ICS</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>Account Age Days</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr"/>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="G89" s="3" t="inlineStr">
+        <is>
+          <t>utils.py</t>
+        </is>
+      </c>
+      <c r="H89" s="3" t="inlineStr">
+        <is>
+          <t>Days since Date Opened</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>ICS</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>Balance Tier</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr"/>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F90" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G90" s="3" t="inlineStr">
+        <is>
+          <t>utils.py</t>
+        </is>
+      </c>
+      <c r="H90" s="3" t="inlineStr">
+        <is>
+          <t>Binned from Curr Bal</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>ICS</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>Age Range</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr"/>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F91" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G91" s="3" t="inlineStr">
+        <is>
+          <t>utils.py</t>
+        </is>
+      </c>
+      <c r="H91" s="3" t="inlineStr">
+        <is>
+          <t>Binned from Account Age Days</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>ICS Append</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>ICS Account</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr"/>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F92" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G92" s="3" t="inlineStr">
+        <is>
+          <t>matcher.py</t>
+        </is>
+      </c>
+      <c r="H92" s="3" t="inlineStr">
+        <is>
+          <t>Yes / No (appended to ODD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>ICS Append</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>ICS Source</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr"/>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F93" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G93" s="3" t="inlineStr">
+        <is>
+          <t>matcher.py</t>
+        </is>
+      </c>
+      <c r="H93" s="3" t="inlineStr">
+        <is>
+          <t>REF / DM / Both / empty</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>ICS Append</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>Acct Hash</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr"/>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G94" s="3" t="inlineStr">
+        <is>
+          <t>merger.py</t>
+        </is>
+      </c>
+      <c r="H94" s="3" t="inlineStr">
+        <is>
+          <t>Normalized account hash from REF/DM files</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>ICS Referral</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>Referrer Name</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>referrer, referrer_name</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F95" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G95" s="3" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="H95" s="3" t="inlineStr">
+        <is>
+          <t>Person who made the referral</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>ICS Referral</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>Issue Date</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>issue_date, date</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="inlineStr">
+        <is>
+          <t>datetime</t>
+        </is>
+      </c>
+      <c r="G96" s="3" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="H96" s="3" t="inlineStr">
+        <is>
+          <t>Referral issue date</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>ICS Referral</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>Referral Code</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>referral_code, code</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F97" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G97" s="3" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="H97" s="3" t="inlineStr">
+        <is>
+          <t>Referral code identifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>ICS Referral</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>Purchase Manager</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>purchase_manager, staff</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F98" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G98" s="3" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="H98" s="3" t="inlineStr">
+        <is>
+          <t>Staff member / purchase manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>ICS Referral</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>branch_id</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F99" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G99" s="3" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="H99" s="3" t="inlineStr">
+        <is>
+          <t>Branch identifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>ICS Referral</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>Account Holder</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>account_holder, new_account</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F100" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G100" s="3" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="H100" s="3" t="inlineStr">
+        <is>
+          <t>New account holder name</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>ICS Referral</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>MRDB Account Hash</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>mrdb_account_hash, mrdb, account_hash</t>
+        </is>
+      </c>
+      <c r="E101" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F101" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G101" s="3" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="H101" s="3" t="inlineStr">
+        <is>
+          <t>Account hash for matching</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>ICS Referral</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>Cert ID</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>cert_id, certificate_id</t>
+        </is>
+      </c>
+      <c r="E102" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F102" s="3" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="G102" s="3" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="H102" s="3" t="inlineStr">
+        <is>
+          <t>Certificate identifier</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H102"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>